<commit_message>
revise if miss transaction id & Test no of FTU and LTX
- ltx reconcile
- expected-case-builder
-summary/automation-summary-writer
</commit_message>
<xml_diff>
--- a/template/DS_FTU_Automation_Summary.xlsx
+++ b/template/DS_FTU_Automation_Summary.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="24" documentId="8_{135E3321-2B5A-4F74-A3E1-AA01D1EDE02D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E30C4791-31BD-50F1-9FA9-AEE4B55DF9A2}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="8_{135E3321-2B5A-4F74-A3E1-AA01D1EDE02D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80EC5E9D-E5FE-44BB-B184-1646CB3DF815}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -14,6 +14,8 @@
     <sheet name="Test Data" sheetId="6" r:id="rId4"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">DS_FTU!$A$1:$BJ$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">DS_FTU_Reconcile!$A$1:$AC$1</definedName>
     <definedName name="_xlnm._FilterDatabase">DS_FTU!$A$1:$BJ$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -34,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="154">
   <si>
     <t>Report File Name:</t>
   </si>
@@ -436,6 +438,66 @@
   </si>
   <si>
     <t>BOT Purpose code</t>
+  </si>
+  <si>
+    <t>Test Result.</t>
+  </si>
+  <si>
+    <t>Dept Code</t>
+  </si>
+  <si>
+    <t>System Id</t>
+  </si>
+  <si>
+    <t>Reference Transaction Number</t>
+  </si>
+  <si>
+    <t>Cust Code</t>
+  </si>
+  <si>
+    <t>CMF CODE</t>
+  </si>
+  <si>
+    <t>Cust Name</t>
+  </si>
+  <si>
+    <t>Data Provider Branch Number</t>
+  </si>
+  <si>
+    <t>FI Reporting Group Id</t>
+  </si>
+  <si>
+    <t>Data Submission Period</t>
+  </si>
+  <si>
+    <t>FX Arrangement Type</t>
+  </si>
+  <si>
+    <t>FX Arrangement Type Name</t>
+  </si>
+  <si>
+    <t>Country Id of Beneficiary Involved Party</t>
+  </si>
+  <si>
+    <t>Country Id of Beneficiary Involved Party Name</t>
+  </si>
+  <si>
+    <t>Business Type of Exercising Involved Party</t>
+  </si>
+  <si>
+    <t>Business Type of Exercising Involved Party Name</t>
+  </si>
+  <si>
+    <t>Inflow Transaction Purpose Name</t>
+  </si>
+  <si>
+    <t>Outflow Transaction Purpose Name</t>
+  </si>
+  <si>
+    <t>Currency Id Name</t>
+  </si>
+  <si>
+    <t>Leg Type Name</t>
   </si>
 </sst>
 </file>
@@ -653,7 +715,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="22">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -757,6 +819,21 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="27">
     <border>
@@ -1243,11 +1320,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1311,6 +1383,11 @@
     <xf numFmtId="0" fontId="21" fillId="11" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1654,30 +1731,30 @@
       <c r="K1" s="6"/>
     </row>
     <row r="2" spans="2:20" ht="28.5" customHeight="1">
-      <c r="B2" s="68" t="s">
+      <c r="B2" s="65" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="69"/>
-      <c r="D2" s="69"/>
-      <c r="E2" s="69"/>
-      <c r="F2" s="69"/>
-      <c r="G2" s="69"/>
-      <c r="H2" s="69"/>
-      <c r="I2" s="69"/>
-      <c r="J2" s="69"/>
-      <c r="K2" s="69"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="66"/>
+      <c r="F2" s="66"/>
+      <c r="G2" s="66"/>
+      <c r="H2" s="66"/>
+      <c r="I2" s="66"/>
+      <c r="J2" s="66"/>
+      <c r="K2" s="66"/>
     </row>
     <row r="3" spans="2:20">
-      <c r="B3" s="69"/>
-      <c r="C3" s="69"/>
-      <c r="D3" s="69"/>
-      <c r="E3" s="69"/>
-      <c r="F3" s="69"/>
-      <c r="G3" s="69"/>
-      <c r="H3" s="69"/>
-      <c r="I3" s="69"/>
-      <c r="J3" s="69"/>
-      <c r="K3" s="69"/>
+      <c r="B3" s="66"/>
+      <c r="C3" s="66"/>
+      <c r="D3" s="66"/>
+      <c r="E3" s="66"/>
+      <c r="F3" s="66"/>
+      <c r="G3" s="66"/>
+      <c r="H3" s="66"/>
+      <c r="I3" s="66"/>
+      <c r="J3" s="66"/>
+      <c r="K3" s="66"/>
     </row>
     <row r="4" spans="2:20" outlineLevel="1" collapsed="1">
       <c r="B4" s="4"/>
@@ -1700,16 +1777,16 @@
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
-      <c r="I5" s="72" t="s">
+      <c r="I5" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="J5" s="74" t="s">
+      <c r="J5" s="71" t="s">
         <v>2</v>
       </c>
-      <c r="K5" s="70" t="s">
+      <c r="K5" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="L5" s="71"/>
+      <c r="L5" s="68"/>
     </row>
     <row r="6" spans="2:20" outlineLevel="1" collapsed="1">
       <c r="B6" s="7" t="s">
@@ -1720,10 +1797,10 @@
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
-      <c r="I6" s="73"/>
-      <c r="J6" s="73"/>
-      <c r="K6" s="70"/>
-      <c r="L6" s="71"/>
+      <c r="I6" s="70"/>
+      <c r="J6" s="70"/>
+      <c r="K6" s="67"/>
+      <c r="L6" s="68"/>
     </row>
     <row r="7" spans="2:20" ht="15" customHeight="1" outlineLevel="1" collapsed="1">
       <c r="B7" s="7" t="s">
@@ -1734,10 +1811,10 @@
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
-      <c r="I7" s="77"/>
-      <c r="J7" s="77"/>
-      <c r="K7" s="75"/>
-      <c r="L7" s="76"/>
+      <c r="I7" s="74"/>
+      <c r="J7" s="74"/>
+      <c r="K7" s="72"/>
+      <c r="L7" s="73"/>
     </row>
     <row r="8" spans="2:20" outlineLevel="1" collapsed="1">
       <c r="B8" s="7" t="s">
@@ -1748,10 +1825,10 @@
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
-      <c r="I8" s="73"/>
-      <c r="J8" s="73"/>
-      <c r="K8" s="75"/>
-      <c r="L8" s="76"/>
+      <c r="I8" s="70"/>
+      <c r="J8" s="70"/>
+      <c r="K8" s="72"/>
+      <c r="L8" s="73"/>
     </row>
     <row r="9" spans="2:20" outlineLevel="1" collapsed="1">
       <c r="B9" s="7" t="s">
@@ -1762,10 +1839,10 @@
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
-      <c r="I9" s="73"/>
-      <c r="J9" s="73"/>
-      <c r="K9" s="75"/>
-      <c r="L9" s="76"/>
+      <c r="I9" s="70"/>
+      <c r="J9" s="70"/>
+      <c r="K9" s="72"/>
+      <c r="L9" s="73"/>
     </row>
     <row r="10" spans="2:20" outlineLevel="1" collapsed="1">
       <c r="B10" s="4"/>
@@ -1792,52 +1869,52 @@
       <c r="K11" s="6"/>
     </row>
     <row r="12" spans="2:20" ht="15" customHeight="1" thickBot="1">
-      <c r="B12" s="61" t="s">
+      <c r="B12" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="62"/>
-      <c r="D12" s="62"/>
-      <c r="E12" s="62"/>
-      <c r="F12" s="62"/>
-      <c r="G12" s="62"/>
-      <c r="H12" s="62"/>
-      <c r="I12" s="62"/>
-      <c r="J12" s="62"/>
-      <c r="K12" s="62"/>
-      <c r="L12" s="62"/>
-      <c r="M12" s="62"/>
-      <c r="N12" s="62"/>
-      <c r="O12" s="62"/>
-      <c r="P12" s="62"/>
-      <c r="Q12" s="62"/>
-      <c r="R12" s="62"/>
-      <c r="S12" s="62"/>
-      <c r="T12" s="62"/>
+      <c r="C12" s="59"/>
+      <c r="D12" s="59"/>
+      <c r="E12" s="59"/>
+      <c r="F12" s="59"/>
+      <c r="G12" s="59"/>
+      <c r="H12" s="59"/>
+      <c r="I12" s="59"/>
+      <c r="J12" s="59"/>
+      <c r="K12" s="59"/>
+      <c r="L12" s="59"/>
+      <c r="M12" s="59"/>
+      <c r="N12" s="59"/>
+      <c r="O12" s="59"/>
+      <c r="P12" s="59"/>
+      <c r="Q12" s="59"/>
+      <c r="R12" s="59"/>
+      <c r="S12" s="59"/>
+      <c r="T12" s="59"/>
     </row>
     <row r="13" spans="2:20" ht="21.5" customHeight="1" thickBot="1">
       <c r="B13" s="8"/>
       <c r="C13" s="9"/>
-      <c r="D13" s="63" t="s">
+      <c r="D13" s="60" t="s">
         <v>129</v>
       </c>
-      <c r="E13" s="64"/>
-      <c r="F13" s="64"/>
-      <c r="G13" s="64"/>
-      <c r="H13" s="64"/>
-      <c r="I13" s="64"/>
-      <c r="J13" s="65"/>
+      <c r="E13" s="61"/>
+      <c r="F13" s="61"/>
+      <c r="G13" s="61"/>
+      <c r="H13" s="61"/>
+      <c r="I13" s="61"/>
+      <c r="J13" s="62"/>
       <c r="K13" s="10"/>
-      <c r="L13" s="66" t="s">
+      <c r="L13" s="63" t="s">
         <v>9</v>
       </c>
-      <c r="M13" s="67"/>
-      <c r="N13" s="67"/>
-      <c r="O13" s="67"/>
-      <c r="P13" s="67"/>
-      <c r="Q13" s="67"/>
-      <c r="R13" s="67"/>
-      <c r="S13" s="67"/>
-      <c r="T13" s="67"/>
+      <c r="M13" s="64"/>
+      <c r="N13" s="64"/>
+      <c r="O13" s="64"/>
+      <c r="P13" s="64"/>
+      <c r="Q13" s="64"/>
+      <c r="R13" s="64"/>
+      <c r="S13" s="64"/>
+      <c r="T13" s="64"/>
     </row>
     <row r="14" spans="2:20" s="11" customFormat="1" ht="29" customHeight="1">
       <c r="B14" s="12" t="s">
@@ -2032,7 +2109,7 @@
   <sheetPr codeName="Sheet2">
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
-  <dimension ref="A1:BM1"/>
+  <dimension ref="A1:AC1"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -2091,74 +2168,97 @@
     <col min="65" max="65" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" ht="16" customHeight="1">
-      <c r="A1" s="60"/>
-      <c r="B1" s="60"/>
-      <c r="C1" s="60"/>
-      <c r="D1" s="60"/>
-      <c r="E1" s="60"/>
-      <c r="F1" s="60"/>
-      <c r="G1" s="60"/>
-      <c r="H1" s="60"/>
-      <c r="I1" s="60"/>
-      <c r="J1" s="60"/>
-      <c r="K1" s="60"/>
-      <c r="L1" s="60"/>
-      <c r="M1" s="60"/>
-      <c r="N1" s="60"/>
-      <c r="O1" s="60"/>
-      <c r="P1" s="60"/>
-      <c r="Q1" s="60"/>
-      <c r="R1" s="60"/>
-      <c r="S1" s="60"/>
-      <c r="T1" s="60"/>
-      <c r="U1" s="60"/>
-      <c r="V1" s="60"/>
-      <c r="W1" s="60"/>
-      <c r="X1" s="60"/>
-      <c r="Y1" s="60"/>
-      <c r="Z1" s="60"/>
-      <c r="AA1" s="60"/>
-      <c r="AB1" s="60"/>
-      <c r="AC1" s="60"/>
-      <c r="AD1" s="60"/>
-      <c r="AE1" s="60"/>
-      <c r="AF1" s="60"/>
-      <c r="AG1" s="60"/>
-      <c r="AH1" s="60"/>
-      <c r="AI1" s="60"/>
-      <c r="AJ1" s="60"/>
-      <c r="AK1" s="60"/>
-      <c r="AL1" s="60"/>
-      <c r="AM1" s="60"/>
-      <c r="AN1" s="60"/>
-      <c r="AO1" s="60"/>
-      <c r="AP1" s="60"/>
-      <c r="AQ1" s="60"/>
-      <c r="AR1" s="60"/>
-      <c r="AS1" s="60"/>
-      <c r="AT1" s="60"/>
-      <c r="AU1" s="60"/>
-      <c r="AV1" s="60"/>
-      <c r="AW1" s="60"/>
-      <c r="AX1" s="60"/>
-      <c r="AY1" s="60"/>
-      <c r="AZ1" s="60"/>
-      <c r="BA1" s="60"/>
-      <c r="BB1" s="60"/>
-      <c r="BC1" s="60"/>
-      <c r="BD1" s="60"/>
-      <c r="BE1" s="60"/>
-      <c r="BF1" s="60"/>
-      <c r="BG1" s="60"/>
-      <c r="BH1" s="60"/>
-      <c r="BI1" s="60"/>
-      <c r="BJ1" s="60"/>
-      <c r="BK1" s="60"/>
-      <c r="BL1" s="60"/>
-      <c r="BM1" s="60"/>
+    <row r="1" spans="1:29" ht="25.5" customHeight="1">
+      <c r="A1" s="79" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="79" t="s">
+        <v>134</v>
+      </c>
+      <c r="C1" s="79" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="79" t="s">
+        <v>135</v>
+      </c>
+      <c r="E1" s="79" t="s">
+        <v>136</v>
+      </c>
+      <c r="F1" s="79" t="s">
+        <v>130</v>
+      </c>
+      <c r="G1" s="79" t="s">
+        <v>137</v>
+      </c>
+      <c r="H1" s="79" t="s">
+        <v>138</v>
+      </c>
+      <c r="I1" s="79" t="s">
+        <v>139</v>
+      </c>
+      <c r="J1" s="79" t="s">
+        <v>140</v>
+      </c>
+      <c r="K1" s="79" t="s">
+        <v>141</v>
+      </c>
+      <c r="L1" s="79" t="s">
+        <v>142</v>
+      </c>
+      <c r="M1" s="79" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="79" t="s">
+        <v>143</v>
+      </c>
+      <c r="O1" s="79" t="s">
+        <v>144</v>
+      </c>
+      <c r="P1" s="79" t="s">
+        <v>145</v>
+      </c>
+      <c r="Q1" s="79" t="s">
+        <v>146</v>
+      </c>
+      <c r="R1" s="79" t="s">
+        <v>147</v>
+      </c>
+      <c r="S1" s="79" t="s">
+        <v>148</v>
+      </c>
+      <c r="T1" s="79" t="s">
+        <v>149</v>
+      </c>
+      <c r="U1" s="79" t="s">
+        <v>28</v>
+      </c>
+      <c r="V1" s="79" t="s">
+        <v>150</v>
+      </c>
+      <c r="W1" s="79" t="s">
+        <v>29</v>
+      </c>
+      <c r="X1" s="79" t="s">
+        <v>151</v>
+      </c>
+      <c r="Y1" s="79" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z1" s="79" t="s">
+        <v>152</v>
+      </c>
+      <c r="AA1" s="79" t="s">
+        <v>131</v>
+      </c>
+      <c r="AB1" s="79" t="s">
+        <v>153</v>
+      </c>
+      <c r="AC1" s="79" t="s">
+        <v>132</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AC1" xr:uid="{1F98D615-FD6F-400E-BAD1-695E8041768F}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
@@ -2169,7 +2269,7 @@
   <sheetPr codeName="Sheet3">
     <tabColor rgb="FF92D050"/>
   </sheetPr>
-  <dimension ref="A1:BJ1"/>
+  <dimension ref="A1:Z1"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="10.453125" customWidth="1"/>
@@ -2236,71 +2336,88 @@
     <col min="62" max="62" width="11.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:62" ht="25" customHeight="1">
-      <c r="A1" s="58"/>
-      <c r="B1" s="58"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="58"/>
-      <c r="E1" s="58"/>
-      <c r="F1" s="59"/>
-      <c r="G1" s="59"/>
-      <c r="H1" s="59"/>
-      <c r="I1" s="59"/>
-      <c r="J1" s="59"/>
-      <c r="K1" s="59"/>
-      <c r="L1" s="59"/>
-      <c r="M1" s="58"/>
-      <c r="N1" s="59"/>
-      <c r="O1" s="59"/>
-      <c r="P1" s="58"/>
-      <c r="Q1" s="59"/>
-      <c r="R1" s="58"/>
-      <c r="S1" s="59"/>
-      <c r="T1" s="58"/>
-      <c r="U1" s="59"/>
-      <c r="V1" s="58"/>
-      <c r="W1" s="59"/>
-      <c r="X1" s="58"/>
-      <c r="Y1" s="59"/>
-      <c r="Z1" s="58"/>
-      <c r="AA1" s="58"/>
-      <c r="AB1" s="59"/>
-      <c r="AC1" s="58"/>
-      <c r="AD1" s="58"/>
-      <c r="AE1" s="58"/>
-      <c r="AF1" s="59"/>
-      <c r="AG1" s="59"/>
-      <c r="AH1" s="58"/>
-      <c r="AI1" s="58"/>
-      <c r="AJ1" s="58"/>
-      <c r="AK1" s="58"/>
-      <c r="AL1" s="58"/>
-      <c r="AM1" s="59"/>
-      <c r="AN1" s="59"/>
-      <c r="AO1" s="58"/>
-      <c r="AP1" s="59"/>
-      <c r="AQ1" s="58"/>
-      <c r="AR1" s="58"/>
-      <c r="AS1" s="58"/>
-      <c r="AT1" s="58"/>
-      <c r="AU1" s="58"/>
-      <c r="AV1" s="58"/>
-      <c r="AW1" s="58"/>
-      <c r="AX1" s="58"/>
-      <c r="AY1" s="58"/>
-      <c r="AZ1" s="58"/>
-      <c r="BA1" s="58"/>
-      <c r="BB1" s="58"/>
-      <c r="BC1" s="58"/>
-      <c r="BD1" s="58"/>
-      <c r="BE1" s="58"/>
-      <c r="BF1" s="58"/>
-      <c r="BG1" s="58"/>
-      <c r="BH1" s="58"/>
-      <c r="BI1" s="58"/>
-      <c r="BJ1" s="58"/>
+    <row r="1" spans="1:26" ht="25" customHeight="1">
+      <c r="A1" s="80" t="s">
+        <v>135</v>
+      </c>
+      <c r="B1" s="80" t="s">
+        <v>136</v>
+      </c>
+      <c r="C1" s="81" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1" s="80" t="s">
+        <v>137</v>
+      </c>
+      <c r="E1" s="80" t="s">
+        <v>138</v>
+      </c>
+      <c r="F1" s="80" t="s">
+        <v>139</v>
+      </c>
+      <c r="G1" s="80" t="s">
+        <v>140</v>
+      </c>
+      <c r="H1" s="80" t="s">
+        <v>141</v>
+      </c>
+      <c r="I1" s="80" t="s">
+        <v>142</v>
+      </c>
+      <c r="J1" s="81" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="80" t="s">
+        <v>143</v>
+      </c>
+      <c r="L1" s="80" t="s">
+        <v>144</v>
+      </c>
+      <c r="M1" s="80" t="s">
+        <v>145</v>
+      </c>
+      <c r="N1" s="81" t="s">
+        <v>146</v>
+      </c>
+      <c r="O1" s="80" t="s">
+        <v>147</v>
+      </c>
+      <c r="P1" s="80" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q1" s="80" t="s">
+        <v>149</v>
+      </c>
+      <c r="R1" s="81" t="s">
+        <v>28</v>
+      </c>
+      <c r="S1" s="80" t="s">
+        <v>150</v>
+      </c>
+      <c r="T1" s="81" t="s">
+        <v>29</v>
+      </c>
+      <c r="U1" s="80" t="s">
+        <v>151</v>
+      </c>
+      <c r="V1" s="81" t="s">
+        <v>13</v>
+      </c>
+      <c r="W1" s="80" t="s">
+        <v>152</v>
+      </c>
+      <c r="X1" s="81" t="s">
+        <v>131</v>
+      </c>
+      <c r="Y1" s="80" t="s">
+        <v>153</v>
+      </c>
+      <c r="Z1" s="81" t="s">
+        <v>132</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:BJ1" xr:uid="{3087E602-052C-4615-B202-20507170DD7D}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2693,28 +2810,28 @@
       </c>
     </row>
     <row r="4" spans="1:106" s="27" customFormat="1" ht="14.5" customHeight="1">
-      <c r="N4" s="78" t="s">
+      <c r="N4" s="75" t="s">
         <v>33</v>
       </c>
-      <c r="O4" s="79"/>
-      <c r="P4" s="79"/>
-      <c r="Q4" s="79"/>
-      <c r="R4" s="79"/>
-      <c r="S4" s="79"/>
-      <c r="T4" s="79"/>
-      <c r="U4" s="79"/>
-      <c r="V4" s="79"/>
-      <c r="W4" s="79"/>
-      <c r="X4" s="79"/>
-      <c r="Y4" s="79"/>
-      <c r="Z4" s="79"/>
-      <c r="AA4" s="79"/>
-      <c r="AB4" s="79"/>
-      <c r="AC4" s="79"/>
-      <c r="AD4" s="79"/>
-      <c r="AE4" s="79"/>
-      <c r="AF4" s="79"/>
-      <c r="AG4" s="80"/>
+      <c r="O4" s="76"/>
+      <c r="P4" s="76"/>
+      <c r="Q4" s="76"/>
+      <c r="R4" s="76"/>
+      <c r="S4" s="76"/>
+      <c r="T4" s="76"/>
+      <c r="U4" s="76"/>
+      <c r="V4" s="76"/>
+      <c r="W4" s="76"/>
+      <c r="X4" s="76"/>
+      <c r="Y4" s="76"/>
+      <c r="Z4" s="76"/>
+      <c r="AA4" s="76"/>
+      <c r="AB4" s="76"/>
+      <c r="AC4" s="76"/>
+      <c r="AD4" s="76"/>
+      <c r="AE4" s="76"/>
+      <c r="AF4" s="76"/>
+      <c r="AG4" s="77"/>
       <c r="AH4" s="28" t="s">
         <v>34</v>
       </c>
@@ -2787,14 +2904,14 @@
       </c>
       <c r="CT4" s="33"/>
       <c r="CU4" s="33"/>
-      <c r="CW4" s="81" t="s">
+      <c r="CW4" s="78" t="s">
         <v>37</v>
       </c>
-      <c r="CX4" s="81"/>
-      <c r="CY4" s="81"/>
-      <c r="CZ4" s="81"/>
-      <c r="DA4" s="81"/>
-      <c r="DB4" s="81"/>
+      <c r="CX4" s="78"/>
+      <c r="CY4" s="78"/>
+      <c r="CZ4" s="78"/>
+      <c r="DA4" s="78"/>
+      <c r="DB4" s="78"/>
     </row>
     <row r="5" spans="1:106" s="52" customFormat="1" ht="18.75" customHeight="1">
       <c r="A5" s="34"/>

</xml_diff>

<commit_message>
revised template summary FTU and FTU-reconcile
</commit_message>
<xml_diff>
--- a/template/DS_FTU_Automation_Summary.xlsx
+++ b/template/DS_FTU_Automation_Summary.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="36" documentId="8_{135E3321-2B5A-4F74-A3E1-AA01D1EDE02D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80EC5E9D-E5FE-44BB-B184-1646CB3DF815}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="8_{135E3321-2B5A-4F74-A3E1-AA01D1EDE02D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{47AE08A2-2670-43C8-B14B-04042F08EF63}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="196" uniqueCount="153">
   <si>
     <t>Report File Name:</t>
   </si>
@@ -435,9 +435,6 @@
   </si>
   <si>
     <t>Foreign Currency Amount</t>
-  </si>
-  <si>
-    <t>BOT Purpose code</t>
   </si>
   <si>
     <t>Test Result.</t>
@@ -1320,6 +1317,11 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1383,11 +1385,6 @@
     <xf numFmtId="0" fontId="21" fillId="11" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="19" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="20" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1731,30 +1728,30 @@
       <c r="K1" s="6"/>
     </row>
     <row r="2" spans="2:20" ht="28.5" customHeight="1">
-      <c r="B2" s="65" t="s">
+      <c r="B2" s="68" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="66"/>
-      <c r="D2" s="66"/>
-      <c r="E2" s="66"/>
-      <c r="F2" s="66"/>
-      <c r="G2" s="66"/>
-      <c r="H2" s="66"/>
-      <c r="I2" s="66"/>
-      <c r="J2" s="66"/>
-      <c r="K2" s="66"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="69"/>
+      <c r="F2" s="69"/>
+      <c r="G2" s="69"/>
+      <c r="H2" s="69"/>
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
     </row>
     <row r="3" spans="2:20">
-      <c r="B3" s="66"/>
-      <c r="C3" s="66"/>
-      <c r="D3" s="66"/>
-      <c r="E3" s="66"/>
-      <c r="F3" s="66"/>
-      <c r="G3" s="66"/>
-      <c r="H3" s="66"/>
-      <c r="I3" s="66"/>
-      <c r="J3" s="66"/>
-      <c r="K3" s="66"/>
+      <c r="B3" s="69"/>
+      <c r="C3" s="69"/>
+      <c r="D3" s="69"/>
+      <c r="E3" s="69"/>
+      <c r="F3" s="69"/>
+      <c r="G3" s="69"/>
+      <c r="H3" s="69"/>
+      <c r="I3" s="69"/>
+      <c r="J3" s="69"/>
+      <c r="K3" s="69"/>
     </row>
     <row r="4" spans="2:20" outlineLevel="1" collapsed="1">
       <c r="B4" s="4"/>
@@ -1777,16 +1774,16 @@
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
       <c r="H5" s="4"/>
-      <c r="I5" s="69" t="s">
+      <c r="I5" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="J5" s="71" t="s">
+      <c r="J5" s="74" t="s">
         <v>2</v>
       </c>
-      <c r="K5" s="67" t="s">
+      <c r="K5" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="L5" s="68"/>
+      <c r="L5" s="71"/>
     </row>
     <row r="6" spans="2:20" outlineLevel="1" collapsed="1">
       <c r="B6" s="7" t="s">
@@ -1797,10 +1794,10 @@
       <c r="F6" s="4"/>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
-      <c r="I6" s="70"/>
-      <c r="J6" s="70"/>
-      <c r="K6" s="67"/>
-      <c r="L6" s="68"/>
+      <c r="I6" s="73"/>
+      <c r="J6" s="73"/>
+      <c r="K6" s="70"/>
+      <c r="L6" s="71"/>
     </row>
     <row r="7" spans="2:20" ht="15" customHeight="1" outlineLevel="1" collapsed="1">
       <c r="B7" s="7" t="s">
@@ -1811,10 +1808,10 @@
       <c r="F7" s="4"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
-      <c r="I7" s="74"/>
-      <c r="J7" s="74"/>
-      <c r="K7" s="72"/>
-      <c r="L7" s="73"/>
+      <c r="I7" s="77"/>
+      <c r="J7" s="77"/>
+      <c r="K7" s="75"/>
+      <c r="L7" s="76"/>
     </row>
     <row r="8" spans="2:20" outlineLevel="1" collapsed="1">
       <c r="B8" s="7" t="s">
@@ -1825,10 +1822,10 @@
       <c r="F8" s="4"/>
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
-      <c r="I8" s="70"/>
-      <c r="J8" s="70"/>
-      <c r="K8" s="72"/>
-      <c r="L8" s="73"/>
+      <c r="I8" s="73"/>
+      <c r="J8" s="73"/>
+      <c r="K8" s="75"/>
+      <c r="L8" s="76"/>
     </row>
     <row r="9" spans="2:20" outlineLevel="1" collapsed="1">
       <c r="B9" s="7" t="s">
@@ -1839,10 +1836,10 @@
       <c r="F9" s="4"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
-      <c r="I9" s="70"/>
-      <c r="J9" s="70"/>
-      <c r="K9" s="72"/>
-      <c r="L9" s="73"/>
+      <c r="I9" s="73"/>
+      <c r="J9" s="73"/>
+      <c r="K9" s="75"/>
+      <c r="L9" s="76"/>
     </row>
     <row r="10" spans="2:20" outlineLevel="1" collapsed="1">
       <c r="B10" s="4"/>
@@ -1869,52 +1866,52 @@
       <c r="K11" s="6"/>
     </row>
     <row r="12" spans="2:20" ht="15" customHeight="1" thickBot="1">
-      <c r="B12" s="58" t="s">
+      <c r="B12" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="59"/>
-      <c r="D12" s="59"/>
-      <c r="E12" s="59"/>
-      <c r="F12" s="59"/>
-      <c r="G12" s="59"/>
-      <c r="H12" s="59"/>
-      <c r="I12" s="59"/>
-      <c r="J12" s="59"/>
-      <c r="K12" s="59"/>
-      <c r="L12" s="59"/>
-      <c r="M12" s="59"/>
-      <c r="N12" s="59"/>
-      <c r="O12" s="59"/>
-      <c r="P12" s="59"/>
-      <c r="Q12" s="59"/>
-      <c r="R12" s="59"/>
-      <c r="S12" s="59"/>
-      <c r="T12" s="59"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62"/>
+      <c r="E12" s="62"/>
+      <c r="F12" s="62"/>
+      <c r="G12" s="62"/>
+      <c r="H12" s="62"/>
+      <c r="I12" s="62"/>
+      <c r="J12" s="62"/>
+      <c r="K12" s="62"/>
+      <c r="L12" s="62"/>
+      <c r="M12" s="62"/>
+      <c r="N12" s="62"/>
+      <c r="O12" s="62"/>
+      <c r="P12" s="62"/>
+      <c r="Q12" s="62"/>
+      <c r="R12" s="62"/>
+      <c r="S12" s="62"/>
+      <c r="T12" s="62"/>
     </row>
     <row r="13" spans="2:20" ht="21.5" customHeight="1" thickBot="1">
       <c r="B13" s="8"/>
       <c r="C13" s="9"/>
-      <c r="D13" s="60" t="s">
+      <c r="D13" s="63" t="s">
         <v>129</v>
       </c>
-      <c r="E13" s="61"/>
-      <c r="F13" s="61"/>
-      <c r="G13" s="61"/>
-      <c r="H13" s="61"/>
-      <c r="I13" s="61"/>
-      <c r="J13" s="62"/>
+      <c r="E13" s="64"/>
+      <c r="F13" s="64"/>
+      <c r="G13" s="64"/>
+      <c r="H13" s="64"/>
+      <c r="I13" s="64"/>
+      <c r="J13" s="65"/>
       <c r="K13" s="10"/>
-      <c r="L13" s="63" t="s">
+      <c r="L13" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="M13" s="64"/>
-      <c r="N13" s="64"/>
-      <c r="O13" s="64"/>
-      <c r="P13" s="64"/>
-      <c r="Q13" s="64"/>
-      <c r="R13" s="64"/>
-      <c r="S13" s="64"/>
-      <c r="T13" s="64"/>
+      <c r="M13" s="67"/>
+      <c r="N13" s="67"/>
+      <c r="O13" s="67"/>
+      <c r="P13" s="67"/>
+      <c r="Q13" s="67"/>
+      <c r="R13" s="67"/>
+      <c r="S13" s="67"/>
+      <c r="T13" s="67"/>
     </row>
     <row r="14" spans="2:20" s="11" customFormat="1" ht="29" customHeight="1">
       <c r="B14" s="12" t="s">
@@ -1964,7 +1961,7 @@
         <v>78</v>
       </c>
       <c r="R14" s="19" t="s">
-        <v>133</v>
+        <v>57</v>
       </c>
       <c r="S14" s="19" t="s">
         <v>63</v>
@@ -2169,91 +2166,91 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="25.5" customHeight="1">
-      <c r="A1" s="79" t="s">
+      <c r="A1" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="79" t="s">
+      <c r="B1" s="58" t="s">
+        <v>133</v>
+      </c>
+      <c r="C1" s="58" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" s="58" t="s">
         <v>134</v>
       </c>
-      <c r="C1" s="79" t="s">
-        <v>30</v>
-      </c>
-      <c r="D1" s="79" t="s">
+      <c r="E1" s="58" t="s">
         <v>135</v>
       </c>
-      <c r="E1" s="79" t="s">
+      <c r="F1" s="58" t="s">
+        <v>130</v>
+      </c>
+      <c r="G1" s="58" t="s">
         <v>136</v>
       </c>
-      <c r="F1" s="79" t="s">
-        <v>130</v>
-      </c>
-      <c r="G1" s="79" t="s">
+      <c r="H1" s="58" t="s">
         <v>137</v>
       </c>
-      <c r="H1" s="79" t="s">
+      <c r="I1" s="58" t="s">
         <v>138</v>
       </c>
-      <c r="I1" s="79" t="s">
+      <c r="J1" s="58" t="s">
         <v>139</v>
       </c>
-      <c r="J1" s="79" t="s">
+      <c r="K1" s="58" t="s">
         <v>140</v>
       </c>
-      <c r="K1" s="79" t="s">
+      <c r="L1" s="58" t="s">
         <v>141</v>
       </c>
-      <c r="L1" s="79" t="s">
+      <c r="M1" s="58" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="M1" s="79" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="79" t="s">
+      <c r="O1" s="58" t="s">
         <v>143</v>
       </c>
-      <c r="O1" s="79" t="s">
+      <c r="P1" s="58" t="s">
         <v>144</v>
       </c>
-      <c r="P1" s="79" t="s">
+      <c r="Q1" s="58" t="s">
         <v>145</v>
       </c>
-      <c r="Q1" s="79" t="s">
+      <c r="R1" s="58" t="s">
         <v>146</v>
       </c>
-      <c r="R1" s="79" t="s">
+      <c r="S1" s="58" t="s">
         <v>147</v>
       </c>
-      <c r="S1" s="79" t="s">
+      <c r="T1" s="58" t="s">
         <v>148</v>
       </c>
-      <c r="T1" s="79" t="s">
+      <c r="U1" s="58" t="s">
+        <v>28</v>
+      </c>
+      <c r="V1" s="58" t="s">
         <v>149</v>
       </c>
-      <c r="U1" s="79" t="s">
-        <v>28</v>
-      </c>
-      <c r="V1" s="79" t="s">
+      <c r="W1" s="58" t="s">
+        <v>29</v>
+      </c>
+      <c r="X1" s="58" t="s">
         <v>150</v>
       </c>
-      <c r="W1" s="79" t="s">
-        <v>29</v>
-      </c>
-      <c r="X1" s="79" t="s">
+      <c r="Y1" s="58" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z1" s="58" t="s">
         <v>151</v>
       </c>
-      <c r="Y1" s="79" t="s">
-        <v>13</v>
-      </c>
-      <c r="Z1" s="79" t="s">
+      <c r="AA1" s="58" t="s">
+        <v>131</v>
+      </c>
+      <c r="AB1" s="58" t="s">
         <v>152</v>
       </c>
-      <c r="AA1" s="79" t="s">
-        <v>131</v>
-      </c>
-      <c r="AB1" s="79" t="s">
-        <v>153</v>
-      </c>
-      <c r="AC1" s="79" t="s">
+      <c r="AC1" s="58" t="s">
         <v>132</v>
       </c>
     </row>
@@ -2337,82 +2334,82 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="25" customHeight="1">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="59" t="s">
+        <v>134</v>
+      </c>
+      <c r="B1" s="59" t="s">
         <v>135</v>
       </c>
-      <c r="B1" s="80" t="s">
+      <c r="C1" s="60" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1" s="59" t="s">
         <v>136</v>
       </c>
-      <c r="C1" s="81" t="s">
-        <v>130</v>
-      </c>
-      <c r="D1" s="80" t="s">
+      <c r="E1" s="59" t="s">
         <v>137</v>
       </c>
-      <c r="E1" s="80" t="s">
+      <c r="F1" s="59" t="s">
         <v>138</v>
       </c>
-      <c r="F1" s="80" t="s">
+      <c r="G1" s="59" t="s">
         <v>139</v>
       </c>
-      <c r="G1" s="80" t="s">
+      <c r="H1" s="59" t="s">
         <v>140</v>
       </c>
-      <c r="H1" s="80" t="s">
+      <c r="I1" s="59" t="s">
         <v>141</v>
       </c>
-      <c r="I1" s="80" t="s">
+      <c r="J1" s="60" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" s="59" t="s">
         <v>142</v>
       </c>
-      <c r="J1" s="81" t="s">
-        <v>12</v>
-      </c>
-      <c r="K1" s="80" t="s">
+      <c r="L1" s="59" t="s">
         <v>143</v>
       </c>
-      <c r="L1" s="80" t="s">
+      <c r="M1" s="59" t="s">
         <v>144</v>
       </c>
-      <c r="M1" s="80" t="s">
+      <c r="N1" s="60" t="s">
         <v>145</v>
       </c>
-      <c r="N1" s="81" t="s">
+      <c r="O1" s="59" t="s">
         <v>146</v>
       </c>
-      <c r="O1" s="80" t="s">
+      <c r="P1" s="59" t="s">
         <v>147</v>
       </c>
-      <c r="P1" s="80" t="s">
+      <c r="Q1" s="59" t="s">
         <v>148</v>
       </c>
-      <c r="Q1" s="80" t="s">
+      <c r="R1" s="60" t="s">
+        <v>28</v>
+      </c>
+      <c r="S1" s="59" t="s">
         <v>149</v>
       </c>
-      <c r="R1" s="81" t="s">
-        <v>28</v>
-      </c>
-      <c r="S1" s="80" t="s">
+      <c r="T1" s="60" t="s">
+        <v>29</v>
+      </c>
+      <c r="U1" s="59" t="s">
         <v>150</v>
       </c>
-      <c r="T1" s="81" t="s">
-        <v>29</v>
-      </c>
-      <c r="U1" s="80" t="s">
+      <c r="V1" s="60" t="s">
+        <v>13</v>
+      </c>
+      <c r="W1" s="59" t="s">
         <v>151</v>
       </c>
-      <c r="V1" s="81" t="s">
-        <v>13</v>
-      </c>
-      <c r="W1" s="80" t="s">
+      <c r="X1" s="60" t="s">
+        <v>131</v>
+      </c>
+      <c r="Y1" s="59" t="s">
         <v>152</v>
       </c>
-      <c r="X1" s="81" t="s">
-        <v>131</v>
-      </c>
-      <c r="Y1" s="80" t="s">
-        <v>153</v>
-      </c>
-      <c r="Z1" s="81" t="s">
+      <c r="Z1" s="60" t="s">
         <v>132</v>
       </c>
     </row>
@@ -2810,28 +2807,28 @@
       </c>
     </row>
     <row r="4" spans="1:106" s="27" customFormat="1" ht="14.5" customHeight="1">
-      <c r="N4" s="75" t="s">
+      <c r="N4" s="78" t="s">
         <v>33</v>
       </c>
-      <c r="O4" s="76"/>
-      <c r="P4" s="76"/>
-      <c r="Q4" s="76"/>
-      <c r="R4" s="76"/>
-      <c r="S4" s="76"/>
-      <c r="T4" s="76"/>
-      <c r="U4" s="76"/>
-      <c r="V4" s="76"/>
-      <c r="W4" s="76"/>
-      <c r="X4" s="76"/>
-      <c r="Y4" s="76"/>
-      <c r="Z4" s="76"/>
-      <c r="AA4" s="76"/>
-      <c r="AB4" s="76"/>
-      <c r="AC4" s="76"/>
-      <c r="AD4" s="76"/>
-      <c r="AE4" s="76"/>
-      <c r="AF4" s="76"/>
-      <c r="AG4" s="77"/>
+      <c r="O4" s="79"/>
+      <c r="P4" s="79"/>
+      <c r="Q4" s="79"/>
+      <c r="R4" s="79"/>
+      <c r="S4" s="79"/>
+      <c r="T4" s="79"/>
+      <c r="U4" s="79"/>
+      <c r="V4" s="79"/>
+      <c r="W4" s="79"/>
+      <c r="X4" s="79"/>
+      <c r="Y4" s="79"/>
+      <c r="Z4" s="79"/>
+      <c r="AA4" s="79"/>
+      <c r="AB4" s="79"/>
+      <c r="AC4" s="79"/>
+      <c r="AD4" s="79"/>
+      <c r="AE4" s="79"/>
+      <c r="AF4" s="79"/>
+      <c r="AG4" s="80"/>
       <c r="AH4" s="28" t="s">
         <v>34</v>
       </c>
@@ -2904,14 +2901,14 @@
       </c>
       <c r="CT4" s="33"/>
       <c r="CU4" s="33"/>
-      <c r="CW4" s="78" t="s">
+      <c r="CW4" s="81" t="s">
         <v>37</v>
       </c>
-      <c r="CX4" s="78"/>
-      <c r="CY4" s="78"/>
-      <c r="CZ4" s="78"/>
-      <c r="DA4" s="78"/>
-      <c r="DB4" s="78"/>
+      <c r="CX4" s="81"/>
+      <c r="CY4" s="81"/>
+      <c r="CZ4" s="81"/>
+      <c r="DA4" s="81"/>
+      <c r="DB4" s="81"/>
     </row>
     <row r="5" spans="1:106" s="52" customFormat="1" ht="18.75" customHeight="1">
       <c r="A5" s="34"/>

</xml_diff>